<commit_message>
Shopping list: plain quantities only
Per Tim: no on-hand/ordered tracking, no spares math, no meta footer —
just Item | Qty | Pack | Packs | URL | Notes on Totals (sign section
inline, bridge S3 counted once in the 16) and Part | Qty | URL | Notes
per room tab. C3 row ships without a URL rather than an unverified ASIN.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shopping-list.xlsx
+++ b/shopping-list.xlsx
@@ -33,16 +33,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -74,12 +71,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,18 +441,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="72" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="64" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -467,40 +460,25 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>In rooms</t>
+          <t>Qty</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Spares</t>
+          <t>Pack size</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Packs</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Pack size</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Packs to buy</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>On hand / ordered</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -513,74 +491,44 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2" t="n">
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>3-pack</t>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>5 more</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>3 ORDERED (1 pack, 7/18)</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15 rooms + 3 flashed spares (1 spare = the Camp Sign bridge)</t>
+          <t>15 room nodes + 1 sign bridge</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Seeed XIAO ESP32-C3 (puck)</t>
+          <t>Seeed XIAO ESP32-C3</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>YES — spare pool</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Moop pucks only; C3s freed by the S3 fleet decision</t>
+          <t>Moop button pucks — same Seeed store as the S3</t>
         </is>
       </c>
     </row>
@@ -594,34 +542,19 @@
         <v>15</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2-pack</t>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>7 more</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2 ORDERED (1 pack, 7/18)</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ships unconfigured — jumper solder per room-node-audio-plan.md</t>
+          <t>jumper solder per room-node-audio-plan.md</t>
         </is>
       </c>
     </row>
@@ -635,32 +568,17 @@
         <v>15</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
         <v>15</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>pair</t>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
-        <is>
-          <t>15 minus owned</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Some — count your pairs</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
         <is>
           <t>must be the ANALOG-input original (V2 unavailable)</t>
         </is>
@@ -679,31 +597,16 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2-pack</t>
+          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>5 more</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>3 ON HAND</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>11 radar rooms + 2 spares</t>
+          <t>11 radar rooms</t>
         </is>
       </c>
     </row>
@@ -717,34 +620,19 @@
         <v>4</v>
       </c>
       <c r="C7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" t="n">
         <v>2</v>
       </c>
-      <c r="D7" t="n">
-        <v>6</v>
-      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3-pack</t>
+          <t>https://www.amazon.com/dp/B0CLDKMGZR</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2 packs</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2 ON HAND (AITRIP = same board)</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0CLDKMGZR</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Entrance/Exit/Guy Line/VMM + spares</t>
+          <t>Entrance / Exit / Guy Line / VMM</t>
         </is>
       </c>
     </row>
@@ -758,28 +646,17 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>https://www.amazon.com/dp/B0CGNMCTRC</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0CGNMCTRC</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
         <is>
           <t>Cuddle projection tracker (UART1)</t>
         </is>
@@ -795,34 +672,19 @@
         <v>3</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>20-pack</t>
+          <t>https://www.amazon.com/dp/B09N2GG52K</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0 — ORDERED</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>20-pk ordered 7/18</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B09N2GG52K</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Porto knock pads + spares</t>
+          <t>Porto knock pads</t>
         </is>
       </c>
     </row>
@@ -836,28 +698,17 @@
         <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>25-pack</t>
+          <t>https://www.amazon.com/dp/B07Y3ZG1Z1</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B07Y3ZG1Z1</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
         <is>
           <t>piezo bleed resistors</t>
         </is>
@@ -873,34 +724,19 @@
         <v>25</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D11" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>5-pack (5-colour)</t>
+          <t>https://www.amazon.com/dp/B01N11BDX9</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>5 more packs</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>1 pack ORDERED 7/18</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B01N11BDX9</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>games need 24 (Gate 6, DPH 5, Bike 4, NFM 5, Moop 4); on-hand pack = Photo Bomb shutter + spares</t>
+          <t>Gate 6, DPH 5, NFM 5, Bike 4, Moop 4, Photo Bomb shutter 1</t>
         </is>
       </c>
     </row>
@@ -914,71 +750,39 @@
         <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10-pack</t>
+          <t>https://www.amazon.com/dp/B07HKDKZD8</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0 — ORDERED</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>10-pk ordered 7/18</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B07HKDKZD8</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Monkey pedestal + spares</t>
+          <t>Monkey pedestal</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hex 4-button station (existing hardware)</t>
+          <t>Hex 4-button station</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>1</v>
       </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>YES — existing hardware</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>terminates at the Cuddle box</t>
+          <t>wires into the Cuddle box</t>
         </is>
       </c>
     </row>
@@ -991,64 +795,34 @@
       <c r="B14" t="n">
         <v>4</v>
       </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>4 (listing TBD)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>protected cells preferred; XIAO battery pads do the charging</t>
+          <t>protected cells preferred; XIAO battery pads do the charging; LISTING TBD</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>WS2812 pixels x5 (truck lamps)</t>
+          <t>WS2811/WS2812 pixels x5 (truck lamps)</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>1</v>
       </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>from Camp Sign reel spares</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>5 px + spare 74AHCT125 level shifter</t>
+          <t>cut from a sign WS2811 reel</t>
         </is>
       </c>
     </row>
@@ -1061,345 +835,235 @@
       <c r="B16" t="n">
         <v>1</v>
       </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>resistor stock</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
-        <is>
           <t>values in wiring-guides/room-games-plan.md</t>
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>CAMP SIGN (see its tab for the full build)</t>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BTF-LIGHTING WS2811 12V 60LED/m 20px/m IP65 black PCB, 5m reel</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01CNL6LLA</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Camp Sign — 24 letter/logo zones; NFM truck lamps cut from the same reels</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BTF-LIGHTING WS2811 12V 60LED/m 20px/m IP65 black PCB, 5m reel</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="n">
-        <v>4</v>
-      </c>
-      <c r="E19" t="inlineStr"/>
+          <t>SN74AHCT125N quad level shifter DIP-14, 10-pack</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B08R6BCSYC</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B01CNL6LLA</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>$22.99/reel @2026-07-19; 24 letter/logo zones; NFM truck lamps cut from the spares</t>
+          <t>Camp Sign — 3.3V-&gt;5V for the 4 data outputs; socket it</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Seeed XIAO ESP32-S3 (sign DMX bridge)</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>pull from fleet spares</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>MUST be S3: 4 RMT TX = the 4 pixel outputs (C3 has only 2)</t>
+          <t>DIANN 12V-&gt;5V 3A 15W buck converter (potted)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BPRV1K6Q</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Camp Sign — feeds S3 + RS485 module off the 12V rail</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SN74AHCT125N quad level shifter DIP-14, 10-pack</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" t="inlineStr"/>
+          <t>Donner Dfi 2.4G wireless DMX kit (1 TX + 1 RX)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00URFIZZA</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B08R6BCSYC</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>3.3V-&gt;5V for the 4 data outputs; socket it; spares cover the NFM truck</t>
+          <t>Camp Sign — wireless hop from the wired DMX chain end</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>DIANN 12V-&gt;5V 3A 15W buck converter (potted)</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" t="inlineStr"/>
+          <t>HiLetgo TTL&lt;-&gt;RS485 auto-flow module, 5-pack</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B082Y19KV9</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0BPRV1K6Q</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>feeds S3 + RS485 module off the 12V rail</t>
+          <t>Camp Sign — DMX receive into UART1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Donner Dfi 2.4G wireless DMX kit (1 TX + 1 RX)</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" t="inlineStr"/>
+          <t>MAYWILLA XLR 3-pin FEMALE pigtail, bare wire end</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0FFMY896F</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B00URFIZZA</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>$50.99 @2026-07-19; wireless hop from the wired DMX chain end</t>
+          <t>Camp Sign — mates the Dfi RX XLR male output to the module</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HiLetgo TTL&lt;-&gt;RS485 auto-flow module, 5-pack</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" t="inlineStr"/>
+          <t>BTF 3-pin IP65 pigtail pairs, 22AWG 20cm, 5-pack</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01LCV8LGA</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B082Y19KV9</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>DMX receive into UART1; replaces the Waveshare isolated module</t>
+          <t>Camp Sign — strip data interconnects — same brand as the strip so they mate</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MAYWILLA XLR 3-pin FEMALE pigtail, bare wire end</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" t="inlineStr"/>
+          <t>BTF 2-pin IP65 pigtail pairs, 18AWG 20cm</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01LCV97AY</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0FFMY896F</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>mates the Dfi RX XLR male output to the module</t>
+          <t>Camp Sign — power-injection drops every ~8ft of strip</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BTF 3-pin IP65 pigtail pairs, 22AWG 20cm, 5-pack</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" t="inlineStr"/>
+          <t>ABI 12V 500W/42A PSU</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B01LCV8LGA</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>strip data interconnects — same brand as the strip so they mate</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>BTF 2-pin IP65 pigtail pairs, 18AWG 20cm (2 packs)</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B01LCV97AY</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>power-injection drops every ~8ft of strip</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>ABI 12V 500W/42A PSU</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>YES — own both</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>one in a pillar (baffled vent), second = on-site spare</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>THE one shopping list (Tim 2026-07-20): Totals + one tab per room + Camp Sign. Sensors/components only —</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>wire, cases/enclosures, USB/power (banks, cubes, extensions), clamps and the router are deliberately excluded</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>(power topology v5 + those rows: hardware-recommendations.md and git history). Listings verified 2026-07-18/19.</t>
+          <t>Camp Sign — one in a pillar (baffled vent), one on site</t>
         </is>
       </c>
     </row>
@@ -1414,14 +1078,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1437,15 +1100,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1460,13 +1118,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -1481,13 +1138,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -1502,13 +1158,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -1523,13 +1178,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>bay radar</t>
         </is>
@@ -1544,13 +1198,12 @@
       <c r="B6" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01N11BDX9</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B01N11BDX9</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
         <is>
           <t>game: 1 random winner of 5; D0-D4</t>
         </is>
@@ -1567,14 +1220,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1590,15 +1242,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1613,13 +1260,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -1634,13 +1280,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -1655,13 +1300,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -1676,13 +1320,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>bay radar</t>
         </is>
@@ -1697,13 +1340,12 @@
       <c r="B6" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01N11BDX9</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B01N11BDX9</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
         <is>
           <t>game: truck Lights-Out row; resistor-ladder ADC</t>
         </is>
@@ -1712,21 +1354,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WS2812 pixels x5 (truck lamps)</t>
+          <t>WS2811/WS2812 pixels x5 (truck lamps)</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>sign reel spares</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>lamps: 5 px cut from the Camp Sign WS2811 reel spares + spare 74AHCT125</t>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>lamps: cut 5 px from a WS2811 reel + 74AHCT125 shifter</t>
         </is>
       </c>
     </row>
@@ -1739,15 +1375,9 @@
       <c r="B8" t="n">
         <v>1</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>from resistor stock; values in room-games-plan.md</t>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>values in room-games-plan.md</t>
         </is>
       </c>
     </row>
@@ -1762,14 +1392,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1785,15 +1414,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1808,13 +1432,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -1829,13 +1452,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -1850,13 +1472,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -1871,13 +1492,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>bay radar (no trigger designed yet — future spec)</t>
         </is>
@@ -1894,14 +1514,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1917,15 +1536,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1940,13 +1554,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -1961,13 +1574,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -1982,13 +1594,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -2003,13 +1614,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>bay radar</t>
         </is>
@@ -2024,15 +1634,14 @@
       <c r="B6" t="n">
         <v>1</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07HKDKZD8</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B07HKDKZD8</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>silver-monkey pedestal switch (from on-hand 10-pk)</t>
+          <t>silver-monkey pedestal switch</t>
         </is>
       </c>
     </row>
@@ -2047,14 +1656,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2070,15 +1678,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2093,13 +1696,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -2114,13 +1716,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -2135,13 +1736,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -2156,13 +1756,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>bay radar</t>
         </is>
@@ -2177,13 +1776,12 @@
       <c r="B6" t="n">
         <v>4</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01N11BDX9</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B01N11BDX9</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
         <is>
           <t>game: 2x true/false quiz; answer key TBD until sign made</t>
         </is>
@@ -2200,14 +1798,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2223,15 +1820,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2246,13 +1838,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -2267,13 +1858,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -2288,13 +1878,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -2309,13 +1898,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CLDKMGZR</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0CLDKMGZR</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>diagonal across the shaft entry arch</t>
         </is>
@@ -2324,21 +1912,16 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Seeed XIAO ESP32-C3 (puck)</t>
+          <t>Seeed XIAO ESP32-C3</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>4</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>spare pool</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>STANDALONE button pucks (from spare pool, $0)</t>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>standalone button pucks</t>
         </is>
       </c>
     </row>
@@ -2351,13 +1934,12 @@
       <c r="B7" t="n">
         <v>4</v>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01N11BDX9</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B01N11BDX9</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
         <is>
           <t>one per puck, on D1</t>
         </is>
@@ -2372,9 +1954,7 @@
       <c r="B8" t="n">
         <v>4</v>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>puck battery on XIAO pads; always-on, nightly recharge; LISTING TBD</t>
         </is>
@@ -2391,14 +1971,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2414,15 +1993,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2437,13 +2011,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -2458,13 +2031,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -2479,13 +2051,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -2500,13 +2071,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CLDKMGZR</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0CLDKMGZR</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>fires out the FINISH arch</t>
         </is>
@@ -2523,14 +2093,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="72" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2546,15 +2115,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2569,15 +2133,14 @@
       <c r="B2" t="n">
         <v>4</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01CNL6LLA</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B01CNL6LLA</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>$22.99/reel @2026-07-19; 24 letter/logo zones; NFM truck lamps cut from the spares</t>
+          <t>24 letter/logo zones; NFM truck lamps cut from the same reels</t>
         </is>
       </c>
     </row>
@@ -2592,17 +2155,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pull from fleet spares</t>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>MUST be S3: 4 RMT TX = the 4 pixel outputs (C3 has only 2)</t>
+          <t>MUST be S3 (4 RMT TX = the 4 pixel outputs); counted in the Totals S3 line</t>
         </is>
       </c>
     </row>
@@ -2615,15 +2173,14 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B08R6BCSYC</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B08R6BCSYC</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>3.3V-&gt;5V for the 4 data outputs; socket it; spares cover the NFM truck</t>
+          <t>3.3V-&gt;5V for the 4 data outputs; socket it</t>
         </is>
       </c>
     </row>
@@ -2636,13 +2193,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BPRV1K6Q</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0BPRV1K6Q</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>feeds S3 + RS485 module off the 12V rail</t>
         </is>
@@ -2657,15 +2213,14 @@
       <c r="B6" t="n">
         <v>1</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00URFIZZA</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B00URFIZZA</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>$50.99 @2026-07-19; wireless hop from the wired DMX chain end</t>
+          <t>wireless hop from the wired DMX chain end</t>
         </is>
       </c>
     </row>
@@ -2678,15 +2233,14 @@
       <c r="B7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B082Y19KV9</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B082Y19KV9</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>DMX receive into UART1; replaces the Waveshare isolated module</t>
+          <t>DMX receive into UART1</t>
         </is>
       </c>
     </row>
@@ -2699,13 +2253,12 @@
       <c r="B8" t="n">
         <v>1</v>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0FFMY896F</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0FFMY896F</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
         <is>
           <t>mates the Dfi RX XLR male output to the module</t>
         </is>
@@ -2720,13 +2273,12 @@
       <c r="B9" t="n">
         <v>1</v>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01LCV8LGA</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B01LCV8LGA</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
         <is>
           <t>strip data interconnects — same brand as the strip so they mate</t>
         </is>
@@ -2735,19 +2287,18 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BTF 2-pin IP65 pigtail pairs, 18AWG 20cm (2 packs)</t>
+          <t>BTF 2-pin IP65 pigtail pairs, 18AWG 20cm</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>2</v>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01LCV97AY</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B01LCV97AY</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
         <is>
           <t>power-injection drops every ~8ft of strip</t>
         </is>
@@ -2762,15 +2313,9 @@
       <c r="B11" t="n">
         <v>2</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>YES — own both</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>one in a pillar (baffled vent), second = on-site spare</t>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>one in a pillar (baffled vent), one on site</t>
         </is>
       </c>
     </row>
@@ -2785,14 +2330,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2808,15 +2352,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2831,13 +2370,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -2852,13 +2390,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -2873,13 +2410,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -2894,13 +2430,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CLDKMGZR</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0CLDKMGZR</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>fires out the START arch, range gate 2.1m</t>
         </is>
@@ -2917,14 +2452,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2940,15 +2474,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2963,13 +2492,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -2984,13 +2512,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -3005,13 +2532,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -3026,13 +2552,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>bay radar</t>
         </is>
@@ -3049,14 +2574,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3072,15 +2596,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3095,13 +2614,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -3116,13 +2634,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -3137,13 +2654,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -3158,13 +2674,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>doorway radar (GateInspection)</t>
         </is>
@@ -3179,13 +2694,12 @@
       <c r="B6" t="n">
         <v>6</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01N11BDX9</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B01N11BDX9</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
         <is>
           <t>game: two banks of 3, body-press simultaneous; D0-D5; LEDs to 5V rail; PLACEMENT PENDING</t>
         </is>
@@ -3202,14 +2716,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3225,15 +2738,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3248,13 +2756,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -3269,13 +2776,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -3290,13 +2796,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -3311,13 +2816,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CLDKMGZR</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0CLDKMGZR</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>diagonal across the shaft entry arch</t>
         </is>
@@ -3334,14 +2838,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3357,15 +2860,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3380,13 +2878,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -3401,13 +2898,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -3422,13 +2918,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -3443,13 +2938,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>bay radar</t>
         </is>
@@ -3466,14 +2960,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3489,15 +2982,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3512,13 +3000,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -3533,13 +3020,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -3554,13 +3040,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -3575,13 +3060,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>bay radar</t>
         </is>
@@ -3596,15 +3080,14 @@
       <c r="B6" t="n">
         <v>3</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B09N2GG52K</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B09N2GG52K</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>knock pads (from on-hand 20-pk)</t>
+          <t>knock pads</t>
         </is>
       </c>
     </row>
@@ -3617,15 +3100,14 @@
       <c r="B7" t="n">
         <v>3</v>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07Y3ZG1Z1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B07Y3ZG1Z1</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>piezo bleed (1 per disc, from 25-pk)</t>
+          <t>piezo bleed, 1 per disc</t>
         </is>
       </c>
     </row>
@@ -3640,14 +3122,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3663,15 +3144,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3686,13 +3162,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -3707,13 +3182,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -3728,13 +3202,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -3749,13 +3222,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>presence/dwell</t>
         </is>
@@ -3770,13 +3242,12 @@
       <c r="B6" t="n">
         <v>1</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CGNMCTRC</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0CGNMCTRC</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
         <is>
           <t>projection position tracking, UART1</t>
         </is>
@@ -3785,21 +3256,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Hex 4-button station (existing hardware)</t>
+          <t>Hex 4-button station</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>4 arcade buttons terminate at this box (11/11 pins full)</t>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>4 arcade buttons wire into this box (11/11 pins full)</t>
         </is>
       </c>
     </row>
@@ -3814,14 +3279,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3837,15 +3301,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>On hand?</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3860,13 +3319,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>node brain</t>
         </is>
@@ -3881,13 +3339,12 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
         </is>
@@ -3902,13 +3359,12 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>room speaker, mounts off-box below</t>
         </is>
@@ -3923,13 +3379,12 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>bay radar</t>
         </is>
@@ -3944,15 +3399,14 @@
       <c r="B6" t="n">
         <v>1</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01N11BDX9</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B01N11BDX9</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>shutter button (from on-hand 5-pk)</t>
+          <t>shutter button</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DB9 field standard, enclosure port B = DMX cut, BOMs with listings
wiring-guides/dmx-over-wifi.md is the plan of record (spec, per-room pins,
MAX485 wiring, rollout, failure table). db9-field-wiring.md lands the DB9
standard: port A etched field IO (7 wired rooms), port B CUT in every box
as the room's DMX out (2=GND 3=D+ 4=D-, DB9->XLR adapter, 120R terminator);
Gate note for the MCP23017. Enclosure SCAD cuts port B + jackscrew holes,
SVGs re-exported, previews re-rendered (incl. the cuddle variant files from
the caliper pass). Camp sign: Art-Net over WiFi is the primary feed, Dfi
kit demoted to fallback pending the tower WiFi test. Pin map updated (DMX
rows; stale Cuddle hex-station line corrected). shopping-list.xlsx: DMX
rows added with verified Amazon listings, GX-aviation and hex-station rows
reconciled to the DB9 standard, per-room sheets updated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shopping-list.xlsx
+++ b/shopping-list.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Totals" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Entrance" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cop Dodge" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gate" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Guy Line Climb" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Sparkle Pony Room" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Porto Room" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Cuddle Cross" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Photo Bomb Room" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Deep Playa Handshake" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="No Friends Monday" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Temple Room" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Monkey Room" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Bike Lock Room" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Vertical Moop March" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Exit" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Camp Sign" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Totals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entrance" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cop Dodge" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guy Line Climb" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sparkle Pony Room" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Porto Room" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuddle Cross" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photo Bomb Room" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deep Playa Handshake" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="No Friends Monday" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Temple Room" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monkey Room" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bike Lock Room" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vertical Moop March" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exit" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camp Sign" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -772,7 +772,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -781,7 +781,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>wires into the Cuddle box</t>
+          <t>SUPERSEDED by the games plan — Cuddle has no wired inputs (db9-field-wiring.md); do not buy</t>
         </is>
       </c>
     </row>
@@ -848,202 +848,215 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GX16-8 aviation connector (panel + inline plug pair)</t>
+          <t>DB9 FEMALE screw-terminal breakout</t>
         </is>
       </c>
       <c r="B17" t="n">
+        <v>25</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>10 (5M+5F)</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
         <v>5</v>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B09WD2V37T</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Gate / DPH / Bike / NFM / Cuddle — multi-button feed into the node box (floor mount)</t>
+          <t>ANMBEST mixed 10pk w/ jackscrew bolts: 5 packs = 25M+25F — ONE order covers this row AND the male row</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GX12-2 aviation connector (panel + inline plug pair)</t>
+          <t>DB9 MALE screw-terminal breakout</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10 (5M+5F)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B09WD2V37T</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Porto x3, Photo Bomb, Monkey — 2-wire feed into the node box (floor mount)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
+          <t>covered by the female row order (mixed packs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module (DE/RE pins broken out)</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>17</v>
+      </c>
+      <c r="C19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B088Q8TD4V</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>ANMBEST 10pk; DE/RE broken out (tie both high = TX-only). 15 rooms + 2 spares, 2 packs = 20</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BTF-LIGHTING WS2811 12V 60LED/m 20px/m IP65 black PCB, 5m reel</t>
+          <t>DB9 M-F straight-through serial extension cables</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>9</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>9</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B01CNL6LLA</t>
+          <t>https://www.amazon.com/dp/B0C5RCKGDL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Camp Sign — 24 letter/logo zones; NFM truck lamps cut from the same reels</t>
+          <t>PhyinLan 6ft; 10ft = JANSANE B07L5D4DWY — pick lengths per room (port A, db9-field-wiring.md)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SN74AHCT125N quad level shifter DIP-14, 10-pack</t>
+          <t>XLR3 M-F cable, 6ft</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>18</v>
+      </c>
+      <c r="C21" t="n">
+        <v>6</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B08R6BCSYC</t>
+          <t>https://www.amazon.com/dp/B0C5CSMQ7X</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Camp Sign — 3.3V-&gt;5V for the 4 data outputs; socket it</t>
+          <t>EBXYA 6ft 6pk multi-color (color = field ID): 15 cut for DB9-&gt;XLR adapters, 2 whole fixture hops, 1 spare</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>DIANN 12V-&gt;5V 3A 15W buck converter (potted)</t>
+          <t>DMX 120R XLR terminator plug</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>16</v>
+      </c>
+      <c r="C22" t="n">
+        <v>8</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B0BPRV1K6Q</t>
+          <t>https://www.amazon.com/dp/B0GGY454HT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Camp Sign — feeds S3 + RS485 module off the 12V rail</t>
+          <t>CZGOR 3-pin 120R 8pk x2 = 15 room chains + 1 spare</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Donner Dfi 2.4G wireless DMX kit (1 TX + 1 RX)</t>
+          <t>DB9 dust caps (M+F pairs)</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>36</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B00URFIZZA</t>
+          <t>https://www.amazon.com/s?k=db9+dust+cover+cap</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Camp Sign — wireless hop from the wired DMX chain end</t>
+          <t>commodity — any silicone F-port plugs + M-plug covers mix, both ports now</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HiLetgo TTL&lt;-&gt;RS485 auto-flow module, 5-pack</t>
+          <t>MCP23017 I2C expander breakout</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>2</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B082Y19KV9</t>
+          <t>https://www.amazon.com/dp/B07P2H1NZG</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Camp Sign — DMX receive into UART1</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>MAYWILLA XLR 3-pin FEMALE pigtail, bare wire end</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0FFMY896F</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Camp Sign — mates the Dfi RX XLR male output to the module</t>
-        </is>
-      </c>
-    </row>
+          <t>Waveshare (addr DIP -&gt; 0x20); Gate pads (game_gate_hw_mcp.yaml) + 1 spare</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BTF 3-pin IP65 pigtail pairs, 22AWG 20cm, 5-pack</t>
+          <t>BTF-LIGHTING WS2811 12V 60LED/m 20px/m IP65 black PCB, 5m reel</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1052,23 +1065,23 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B01LCV8LGA</t>
+          <t>https://www.amazon.com/dp/B01CNL6LLA</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Camp Sign — strip data interconnects — same brand as the strip so they mate</t>
+          <t>Camp Sign — 24 letter/logo zones; NFM truck lamps cut from the same reels</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>BTF 2-pin IP65 pigtail pairs, 18AWG 20cm</t>
+          <t>SN74AHCT125N quad level shifter DIP-14, 10-pack</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1077,30 +1090,180 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B01LCV97AY</t>
+          <t>https://www.amazon.com/dp/B08R6BCSYC</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Camp Sign — power-injection drops every ~8ft of strip</t>
+          <t>Camp Sign — 3.3V-&gt;5V for the 4 data outputs; socket it</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>DIANN 12V-&gt;5V 3A 15W buck converter (potted)</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BPRV1K6Q</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Camp Sign — feeds S3 + RS485 module off the 12V rail</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Donner Dfi 2.4G wireless DMX kit (1 TX + 1 RX)</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00URFIZZA</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>FALLBACK ONLY (dmx-over-wifi.md): sign primary feed is Art-Net over WiFi — buy/keep only if the tower WiFi fails the on-site test</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>HiLetgo TTL&lt;-&gt;RS485 auto-flow module, 5-pack</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B082Y19KV9</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Camp Sign Dfi-FALLBACK DMX receive only now (dmx-over-wifi.md) — room DMX uses the MAX485 row instead</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MAYWILLA XLR 3-pin FEMALE pigtail, bare wire end</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0FFMY896F</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Camp Sign Dfi-FALLBACK only now (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BTF 3-pin IP65 pigtail pairs, 22AWG 20cm, 5-pack</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01LCV8LGA</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Camp Sign — strip data interconnects — same brand as the strip so they mate</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>BTF 2-pin IP65 pigtail pairs, 18AWG 20cm</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01LCV97AY</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Camp Sign — power-injection drops every ~8ft of strip</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>ABI 12V 500W/42A PSU</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B34" t="n">
         <v>2</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Camp Sign — one in a pillar (baffled vent), one on site</t>
         </is>
@@ -1117,7 +1280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1251,16 +1414,75 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GX16-8 aviation connector (panel + inline plug pair)</t>
+          <t>DB9 port-A field set (F box breakout + M pod breakout + M-F straight cable)</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5 game buttons + common — multi-button feed into the node box (floor mount)</t>
+          <t>port A field IO — replaces the aviation connector (db9-field-wiring.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>
@@ -1270,6 +1492,253 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Seeed XIAO ESP32-S3 (plain, NOT Sense)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>node brain</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PCM5102A I2S DAC board (purple GY-PCM5102)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Creative Pebble 2.0 pair (analog 3.5mm model)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0791H74NT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>room speaker, mounts off-box below</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HLK-LD2410C 24GHz presence radar</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>bay radar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>30mm LED arcade button (EG Starts 5-colour)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01N11BDX9</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>game: truck Lights-Out row; resistor-ladder ADC</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>WS2811/WS2812 pixels x5 (truck lamps)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>lamps: cut 5 px from a WS2811 reel + 74AHCT125 shifter</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Resistor-ladder set (truck buttons)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>values in room-games-plan.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DB9 port-A field set (F box breakout + M pod breakout + M-F straight cable)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>port A field IO — replaces the aviation connector (db9-field-wiring.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1382,34 +1851,29 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>bay radar</t>
+          <t>bay radar (no trigger designed yet — future spec)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>30mm LED arcade button (EG Starts 5-colour)</t>
+          <t>MAX485 TTL-&gt;RS485 module</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B01N11BDX9</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>game: truck Lights-Out row; resistor-ladder ADC</t>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WS2811/WS2812 pixels x5 (truck lamps)</t>
+          <t>DB9 FEMALE screw-terminal breakout</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1417,14 +1881,14 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>lamps: cut 5 px from a WS2811 reel + 74AHCT125 shifter</t>
+          <t>port B (DMX) — bolts into the cut opening</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Resistor-ladder set (truck buttons)</t>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1432,145 +1896,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>values in room-games-plan.md</t>
+          <t>the DB9-&gt;XLR DMX adapter</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GX16-8 aviation connector (panel + inline plug pair)</t>
+          <t>DMX 120R XLR terminator plug</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>1</v>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>5 truck buttons via resistor ladder (2 wires used, spare pins) — multi-button feed into the node box (floor mount)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="78" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Seeed XIAO ESP32-S3 (plain, NOT Sense)</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ6NQFKX</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>node brain</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>PCM5102A I2S DAC board (purple GY-PCM5102)</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DNW32Y46</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>I2S line-out; solder jumpers FLT/DEMP/FMT-&gt;L, XSMT-&gt;H, SCK-&gt;GND</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Creative Pebble 2.0 pair (analog 3.5mm model)</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0791H74NT</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>room speaker, mounts off-box below</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>HLK-LD2410C 24GHz presence radar</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DP9QSQRD</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>bay radar (no trigger designed yet — future spec)</t>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1719,16 +2060,75 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GX12-2 aviation connector (panel + inline plug pair)</t>
+          <t>DB9 port-A field set (F box breakout + M pod breakout + M-F straight cable)</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>pedestal microswitch — 2-wire feed into the node box (floor mount)</t>
+          <t>port A field IO — replaces the aviation connector (db9-field-wiring.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>
@@ -1743,7 +2143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1877,16 +2277,75 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GX16-8 aviation connector (panel + inline plug pair)</t>
+          <t>DB9 port-A field set (F box breakout + M pod breakout + M-F straight cable)</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4 quiz buttons + common — multi-button feed into the node box (floor mount)</t>
+          <t>port A field IO — replaces the aviation connector (db9-field-wiring.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>
@@ -1901,7 +2360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2059,6 +2518,66 @@
       <c r="D8" t="inlineStr">
         <is>
           <t>puck battery on XIAO pads; always-on, nightly recharge; LISTING TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2181,6 +2700,66 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>fires out the FINISH arch</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2418,6 +2997,66 @@
       <c r="D11" t="inlineStr">
         <is>
           <t>one in a pillar (baffled vent), one on site</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>
@@ -2432,7 +3071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2540,6 +3179,66 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>fires out the START arch, range gate 2.1m</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>
@@ -2554,7 +3253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2662,6 +3361,66 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>bay radar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>
@@ -2676,7 +3435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2803,23 +3562,97 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>game: two banks of 3, body-press simultaneous; D0-D5; LEDs to 5V rail; PLACEMENT PENDING</t>
+          <t>game: two banks of 3, body-press simultaneous; MCP23017 GPA0-5 (pin-full after DMX — game_gate_hw_mcp.yaml); LEDs to 5V rail; PLACEMENT PENDING</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GX16-8 aviation connector (panel + inline plug pair)</t>
+          <t>DB9 port-A field set (F box breakout + M pod breakout + M-F straight cable)</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6 game pads + common — multi-button feed into the node box (floor mount)</t>
+          <t>port A field IO — replaces the aviation connector (db9-field-wiring.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MCP23017 I2C expander breakout</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>pads move here (pin-full) — I2C D4/D5, game_gate_hw_mcp.yaml</t>
         </is>
       </c>
     </row>
@@ -2834,7 +3667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2942,6 +3775,66 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>diagonal across the shaft entry arch</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>
@@ -2956,7 +3849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3064,6 +3957,66 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>bay radar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>
@@ -3078,7 +4031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3232,16 +4185,75 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GX12-2 aviation connector (panel + inline plug pair)</t>
+          <t>DB9 port-A field set (F box breakout + M pod breakout + M-F straight cable)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>one per piezo knock pad — 2-wire feed into the node box (floor mount)</t>
+          <t>port A field IO — replaces the aviation connector (db9-field-wiring.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>
@@ -3256,7 +4268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3394,11 +4406,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4 arcade buttons wire into this box (11/11 pins full)</t>
+          <t>SUPERSEDED by the games plan — no Cuddle wired inputs; do not buy</t>
         </is>
       </c>
     </row>
@@ -3409,12 +4421,71 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
+        <v>0</v>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>hex 4-button station + common — multi-button feed into the node box (floor mount)</t>
+          <t>SUPERSEDED — Cuddle has no wired inputs (games plan / db9-field-wiring.md); do not buy</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>
@@ -3429,7 +4500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3563,16 +4634,75 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GX12-2 aviation connector (panel + inline plug pair)</t>
+          <t>DB9 port-A field set (F box breakout + M pod breakout + M-F straight cable)</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>shutter button — 2-wire feed into the node box (floor mount)</t>
+          <t>port A field IO — replaces the aviation connector (db9-field-wiring.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MAX485 TTL-&gt;RS485 module</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DMX out driver — DE/RE tied high (dmx-over-wifi.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DB9 FEMALE screw-terminal breakout</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>port B (DMX) — bolts into the cut opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DB9 MALE screw-terminal breakout + cut XLR3 cable</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>the DB9-&gt;XLR DMX adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DMX 120R XLR terminator plug</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>last fixture OUT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NFM truck: lamps-from-stash + the missing hardware glue
Tim confirmed the wooden truck model is real and the lamps come from his
strip stash - any 5V addressable (WS2812B/SK6812), never 12V sign-reel
stock (DB9-A pins 1/2 supply 5V). game_lightsout_hw.yaml is the
hardware-flash companion the plan promised but never provided: renders
the game bitmask to the 5-px chain (50ms addressable lambda, chipset/
rgb_order substitutions for whatever strip gets grabbed) and decodes the
button ladder on the D0 ADC with 2-sample confirmation. The dangling
"ladder values in room-games-plan.md" reference now resolves: 10k top +
0R/2.2k/4.7k/10k/22k (~0.5V spacing). 74AHCT125 documented in-box so
pin 4 carries 5V-level data down the cable. BOM rows updated (pixels =
$0 from stash, sign reels no longer feed the truck). NFM hardware stack
config-validates; host room sweep still green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shopping-list.xlsx
+++ b/shopping-list.xlsx
@@ -808,11 +808,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>WS2811/WS2812 pixels x5 (truck lamps)</t>
+          <t>5V addressable pixels x5 (NFM truck lamps)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -821,7 +821,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>cut from a sign WS2811 reel</t>
+          <t>FROM TIM'S STASH - any 5V WS2812B/SK6812 strip, NOT 12V sign stock (DB9 supplies 5V); set truck_chipset/truck_rgb_order at flash (game_lightsout_hw.yaml)</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>values in wiring-guides/room-games-plan.md</t>
+          <t>10k top + 0R/2.2k/4.7k/10k/22k per button - values now IN room-games-plan.md + game_lightsout_hw.yaml</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Camp Sign — 24 letter/logo zones; NFM truck lamps cut from the same reels</t>
+          <t>Camp Sign - 24 letter/logo zones (NFM truck lamps now from stash, not these reels)</t>
         </is>
       </c>
     </row>
@@ -1631,15 +1631,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WS2811/WS2812 pixels x5 (truck lamps)</t>
+          <t>5V addressable pixels x5 (truck lamps)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>lamps: cut 5 px from a WS2811 reel + 74AHCT125 shifter</t>
+          <t>FROM STASH - any 5V WS2812B/SK6812, NOT 12V; chipset/order set at flash</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>values in room-games-plan.md</t>
+          <t>10k top + 0R/2.2k/4.7k/10k/22k (room-games-plan.md); + 74AHCT125 from sign spares, in-box</t>
         </is>
       </c>
     </row>

</xml_diff>